<commit_message>
1. modify datases.xlsx to remove some useless index. 2. modify sql generate logic. 3. modify design documents.
</commit_message>
<xml_diff>
--- a/documents/database/databases.xlsx
+++ b/documents/database/databases.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/445c6c4e8400985e/win数据迁移/Projects/Expense Statistics App Project/documents/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="337" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{703E4B94-6434-48EE-83AD-DB90F4DEEBBA}"/>
+  <xr:revisionPtr revIDLastSave="369" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6BE0F26-EFAA-4263-92CC-1F7119BB4686}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6660" yWindow="2124" windowWidth="19572" windowHeight="13872" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_users" sheetId="1" r:id="rId1"/>
     <sheet name="02_account_books" sheetId="2" r:id="rId2"/>
-    <sheet name="03_account_to_users" sheetId="4" r:id="rId3"/>
+    <sheet name="03_accountbook_user_permissions" sheetId="4" r:id="rId3"/>
     <sheet name="04_account_invitations" sheetId="6" r:id="rId4"/>
     <sheet name="05_expense_categories" sheetId="7" r:id="rId5"/>
     <sheet name="06_expenses" sheetId="8" r:id="rId6"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="604" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="142">
   <si>
     <t>Table name：</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -175,10 +175,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>own_user_id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>index on users(id)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -188,9 +184,6 @@
   </si>
   <si>
     <t>NULL</t>
-  </si>
-  <si>
-    <t>account_to_users</t>
   </si>
   <si>
     <t>user_id</t>
@@ -394,9 +387,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>auth_refresh_tokens</t>
-  </si>
-  <si>
     <t>refresh_token</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -441,10 +431,6 @@
   </si>
   <si>
     <t>"user"</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>"CNY"</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -650,6 +636,22 @@
   </si>
   <si>
     <t>DATE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>accountbook_user_permissions</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>owner_user_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>maybe we can add index.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>auth_refresh_tokens</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1089,19 +1091,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1118,13 +1120,10 @@
         <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
@@ -1143,9 +1142,6 @@
       <c r="G4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
@@ -1190,7 +1186,7 @@
       </c>
       <c r="H7" s="3"/>
       <c r="L7" s="1" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1198,7 +1194,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>17</v>
@@ -1207,10 +1203,10 @@
         <v>14</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="M8" s="3"/>
     </row>
@@ -1219,7 +1215,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -1230,11 +1226,8 @@
       <c r="F9" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="I9" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="J9" s="1" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1248,7 +1241,7 @@
         <v>23</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="H10" s="1" t="b">
         <v>1</v>
@@ -1352,7 +1345,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>85</v>
+        <v>141</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1381,19 +1374,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1421,7 +1414,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -1435,11 +1428,9 @@
       <c r="G4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -1449,7 +1440,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>17</v>
@@ -1457,7 +1448,9 @@
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>87</v>
+      </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -1468,7 +1461,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>25</v>
@@ -1488,7 +1481,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>25</v>
@@ -1514,6 +1507,9 @@
       </c>
       <c r="F8" s="2" t="s">
         <v>14</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>26</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -1563,7 +1559,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1592,19 +1588,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1632,7 +1628,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -1647,7 +1643,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -1657,7 +1653,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>17</v>
@@ -1676,13 +1672,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -1690,7 +1686,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>12</v>
@@ -1711,10 +1707,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>13</v>
@@ -1730,10 +1726,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>14</v>
@@ -1744,7 +1740,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>17</v>
@@ -1863,19 +1859,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>116</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>120</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1897,9 +1893,6 @@
       <c r="H3" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="6" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
@@ -1920,7 +1913,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>32</v>
+        <v>139</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -1932,10 +1925,10 @@
         <v>14</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -1943,7 +1936,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>21</v>
@@ -1951,11 +1944,9 @@
       <c r="F6" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="9" t="s">
-        <v>98</v>
-      </c>
+      <c r="H6" s="9"/>
       <c r="L6" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2037,7 +2028,7 @@
         <v>13</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2082,7 +2073,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>36</v>
+        <v>138</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2111,19 +2102,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2151,7 +2142,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2162,17 +2153,15 @@
       <c r="F4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="G4" s="2"/>
       <c r="I4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2180,7 +2169,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -2191,17 +2180,15 @@
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G5" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="G5" s="2"/>
       <c r="I5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -2209,7 +2196,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -2218,10 +2205,10 @@
         <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2243,12 +2230,12 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2293,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2322,19 +2309,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2362,7 +2349,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>12</v>
@@ -2373,11 +2360,8 @@
       <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="J4" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2385,7 +2369,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -2396,11 +2380,8 @@
       <c r="F5" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="6" t="s">
-        <v>13</v>
-      </c>
       <c r="J5" s="6" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2408,7 +2389,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>17</v>
@@ -2417,10 +2398,10 @@
         <v>14</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2428,7 +2409,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>17</v>
@@ -2441,7 +2422,7 @@
       </c>
       <c r="H7" s="7"/>
       <c r="M7" s="7" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2449,7 +2430,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>25</v>
@@ -2466,10 +2447,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F9" s="6" t="s">
         <v>14</v>
@@ -2480,10 +2461,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>14</v>
@@ -2494,19 +2475,19 @@
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="F11" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2568,7 +2549,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2597,19 +2578,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2631,16 +2612,13 @@
       <c r="H3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>13</v>
-      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2655,10 +2633,10 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2694,7 +2672,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>23</v>
@@ -2754,7 +2732,7 @@
         <v>13</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -2799,7 +2777,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2839,19 +2817,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2875,9 +2853,7 @@
       <c r="H3" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="I3" s="1"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
@@ -2888,7 +2864,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2906,7 +2882,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2917,7 +2893,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -2931,11 +2907,9 @@
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2946,7 +2920,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>12</v>
@@ -2964,7 +2938,7 @@
         <v>13</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2975,7 +2949,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>12</v>
@@ -2993,7 +2967,7 @@
         <v>13</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -3050,10 +3024,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -3073,7 +3047,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
@@ -3089,7 +3063,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="M11" s="1"/>
     </row>
@@ -3098,10 +3072,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -3121,10 +3095,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -3144,10 +3118,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -3231,7 +3205,7 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -3281,7 +3255,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3310,19 +3284,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3350,7 +3324,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -3365,7 +3339,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3373,7 +3347,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -3384,14 +3358,11 @@
       <c r="F5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="I5" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="J5" s="1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3399,7 +3370,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -3408,10 +3379,10 @@
         <v>14</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.45">
@@ -3419,19 +3390,19 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="F7" s="1" t="s">
         <v>62</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>64</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
       <c r="M7" s="11" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3439,10 +3410,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>14</v>
@@ -3453,16 +3424,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3479,7 +3450,7 @@
         <v>14</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3487,7 +3458,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>25</v>
@@ -3501,7 +3472,7 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>25</v>
@@ -3586,7 +3557,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3615,19 +3586,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3655,7 +3626,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -3669,7 +3640,7 @@
       <c r="J4" s="2"/>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3677,7 +3648,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -3691,7 +3662,7 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -3699,16 +3670,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="11" t="s">
         <v>73</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>74</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3716,10 +3687,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>14</v>
@@ -3753,12 +3724,12 @@
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>
@@ -3803,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3832,19 +3803,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3872,7 +3843,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -3887,12 +3858,12 @@
         <v>13</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3900,30 +3871,30 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>131</v>
-      </c>
-      <c r="M5" s="6"/>
+        <v>127</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>17</v>
@@ -3937,7 +3908,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>17</v>
@@ -3955,26 +3926,26 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="13" t="s">
-        <v>132</v>
-      </c>
-      <c r="M8" s="6"/>
+        <v>128</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>140</v>
+      </c>
     </row>
     <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A9" s="4">

</xml_diff>

<commit_message>
1. Finished all models and repositories. 2. Changed exchange_rates.date to exchange_rates.rate_date. Add Composite Unique for exchange_rates table. 3. Changed some file names.
But not all tested.
</commit_message>
<xml_diff>
--- a/documents/database/databases.xlsx
+++ b/documents/database/databases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/445c6c4e8400985e/win数据迁移/Projects/Expense Statistics App Project/documents/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="369" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A6BE0F26-EFAA-4263-92CC-1F7119BB4686}"/>
+  <xr:revisionPtr revIDLastSave="379" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9BFD7E38-B850-4B7B-9344-FC4A424629CC}"/>
   <bookViews>
-    <workbookView xWindow="6660" yWindow="2124" windowWidth="19572" windowHeight="13872" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="4" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_users" sheetId="1" r:id="rId1"/>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="593" uniqueCount="144">
   <si>
     <t>Table name：</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -352,10 +352,6 @@
     <t>rate = base_currency / target_currency</t>
   </si>
   <si>
-    <t>date</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>others:</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -654,12 +650,58 @@
     <t>auth_refresh_tokens</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>user_id is Unique now, if we want to support login an account on multiple devices. Just remove Unique</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>cuq_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>exchange_rate</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <family val="3"/>
+        <charset val="134"/>
+      </rPr>
+      <t>_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>date</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -715,6 +757,13 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
       <family val="3"/>
       <charset val="134"/>
     </font>
@@ -1091,19 +1140,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1186,7 +1235,7 @@
       </c>
       <c r="H7" s="3"/>
       <c r="L7" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1194,7 +1243,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>17</v>
@@ -1203,10 +1252,10 @@
         <v>14</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="M8" s="3"/>
     </row>
@@ -1215,7 +1264,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -1227,7 +1276,7 @@
         <v>13</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1345,7 +1394,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1374,19 +1423,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1430,17 +1479,20 @@
       </c>
       <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
+      <c r="M4" s="1" t="s">
+        <v>141</v>
+      </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A5" s="4">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>17</v>
@@ -1449,7 +1501,7 @@
         <v>14</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
@@ -1481,7 +1533,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>25</v>
@@ -1559,7 +1611,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1588,19 +1640,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1643,7 +1695,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -1653,7 +1705,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>17</v>
@@ -1672,13 +1724,13 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -1686,7 +1738,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>12</v>
@@ -1707,10 +1759,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C8" s="10" t="s">
         <v>89</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>90</v>
       </c>
       <c r="F8" s="2" t="s">
         <v>13</v>
@@ -1726,10 +1778,10 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>14</v>
@@ -1740,7 +1792,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>17</v>
@@ -1859,19 +1911,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K2" s="6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L2" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M2" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1913,7 +1965,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -1925,10 +1977,10 @@
         <v>14</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -1946,7 +1998,7 @@
       </c>
       <c r="H6" s="9"/>
       <c r="L6" s="6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2073,7 +2125,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2102,19 +2154,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2142,7 +2194,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2158,10 +2210,10 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2185,10 +2237,10 @@
         <v>13</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -2196,7 +2248,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -2205,10 +2257,10 @@
         <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2235,7 +2287,7 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
   </sheetData>
@@ -2309,19 +2361,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2349,7 +2401,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>12</v>
@@ -2361,7 +2413,7 @@
         <v>14</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2381,7 +2433,7 @@
         <v>14</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2389,7 +2441,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>17</v>
@@ -2398,10 +2450,10 @@
         <v>14</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2484,10 +2536,10 @@
         <v>14</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2578,19 +2630,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2618,7 +2670,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2633,10 +2685,10 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -2817,19 +2869,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2864,7 +2916,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2882,7 +2934,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -2909,7 +2961,7 @@
       <c r="H5" s="1"/>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
@@ -2938,7 +2990,7 @@
         <v>13</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -2967,7 +3019,7 @@
         <v>13</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -3063,7 +3115,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="M11" s="1"/>
     </row>
@@ -3121,7 +3173,7 @@
         <v>58</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -3284,19 +3336,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3324,7 +3376,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -3339,7 +3391,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3359,10 +3411,10 @@
         <v>13</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3370,7 +3422,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -3379,10 +3431,10 @@
         <v>14</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.45">
@@ -3433,7 +3485,7 @@
         <v>62</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3450,7 +3502,7 @@
         <v>14</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3546,7 +3598,7 @@
     <col min="8" max="8" width="19" style="1" customWidth="1"/>
     <col min="9" max="9" width="6.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="32.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.109375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="19.21875" style="1" customWidth="1"/>
     <col min="12" max="12" width="22.44140625" style="1" customWidth="1"/>
     <col min="13" max="13" width="32.21875" style="1" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="1"/>
@@ -3586,19 +3638,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>112</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3634,13 +3686,13 @@
       <c r="F4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
+      <c r="K4" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="L4" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3656,13 +3708,13 @@
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="I5" s="2"/>
       <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
+      <c r="K5" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="L5" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -3687,10 +3739,10 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>74</v>
+        <v>143</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>14</v>
@@ -3698,11 +3750,11 @@
       <c r="H7" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="I7" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="I7" s="2"/>
       <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
+      <c r="K7" s="2" t="s">
+        <v>142</v>
+      </c>
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3724,12 +3776,12 @@
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A11" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -3774,7 +3826,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3803,19 +3855,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="M2" s="1" t="s">
         <v>114</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3858,7 +3910,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
@@ -3871,10 +3923,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="10" t="s">
         <v>78</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>79</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>14</v>
@@ -3883,10 +3935,10 @@
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="M5" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3894,7 +3946,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>17</v>
@@ -3908,7 +3960,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>17</v>
@@ -3929,22 +3981,22 @@
         <v>45</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H8" s="12" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
       <c r="K8" s="2"/>
       <c r="L8" s="13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="M8" s="6" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
revised the sql generate tool's code and databases.xlsx
1.revised sql generate tool to support "other:" for extra constraint.
2.revised databases.xlsx and sql_summary.sql:
	1.make accountbook_user_permissions table be the only truth,
	owner_id of account_books table will be a cache.
	2.account_invitations: the invitation can be multi-used.
	3.now expense_categories.account_book_id can not be NULL. The
	initial categories for users are in a new table called category_templates.
	4.auth_refresh_tokens.user_id is not unique now. For
	multi-device login.
	5.Split request_logs and audit_events
</commit_message>
<xml_diff>
--- a/documents/database/databases.xlsx
+++ b/documents/database/databases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/445c6c4e8400985e/win数据迁移/Projects/Expense Statistics App Project/documents/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="528" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D5BA10A5-1CD8-4BFE-A4DB-164D808A5896}"/>
+  <xr:revisionPtr revIDLastSave="703" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF85CBA6-8540-4A6A-8708-14D2FF62399D}"/>
   <bookViews>
-    <workbookView xWindow="1308" yWindow="2112" windowWidth="22092" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="420" windowWidth="20604" windowHeight="15804" firstSheet="7" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_users" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,16 @@
     <sheet name="03_accountbook_user_permissions" sheetId="4" r:id="rId3"/>
     <sheet name="04_account_invitations" sheetId="6" r:id="rId4"/>
     <sheet name="05_expense_categories" sheetId="7" r:id="rId5"/>
-    <sheet name="06_expenses" sheetId="8" r:id="rId6"/>
-    <sheet name="07_budgets" sheetId="10" r:id="rId7"/>
-    <sheet name="08_exchange_rates" sheetId="11" r:id="rId8"/>
-    <sheet name="09_notifications" sheetId="12" r:id="rId9"/>
-    <sheet name="10_auth_refresh_tokens" sheetId="13" r:id="rId10"/>
-    <sheet name="11_audit_log" sheetId="16" r:id="rId11"/>
-    <sheet name="12_verification_session" sheetId="19" r:id="rId12"/>
-    <sheet name="temp" sheetId="17" r:id="rId13"/>
+    <sheet name="06_category_templates" sheetId="23" r:id="rId6"/>
+    <sheet name="07_expenses" sheetId="8" r:id="rId7"/>
+    <sheet name="08_budgets" sheetId="10" r:id="rId8"/>
+    <sheet name="09_exchange_rates" sheetId="11" r:id="rId9"/>
+    <sheet name="10_notifications" sheetId="12" r:id="rId10"/>
+    <sheet name="11_auth_refresh_tokens" sheetId="13" r:id="rId11"/>
+    <sheet name="12_request_logs" sheetId="16" r:id="rId12"/>
+    <sheet name="13_audit_events" sheetId="24" r:id="rId13"/>
+    <sheet name="14_email_verification" sheetId="19" r:id="rId14"/>
+    <sheet name="temp" sheetId="17" r:id="rId15"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="671" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="192">
   <si>
     <t>Table name：</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -167,9 +169,6 @@
   <si>
     <t>NULL</t>
     <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t xml:space="preserve">UNIQUE INDEX users_email_unique (email); </t>
   </si>
   <si>
     <t>account_books</t>
@@ -353,14 +352,6 @@
     <t>rate = base_currency / target_currency</t>
   </si>
   <si>
-    <t>others:</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>CREATE UNIQUE INDEX idx_rate_unique ON exchange_rates(base_currency, target_currency, date);</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>notifications</t>
   </si>
   <si>
@@ -411,18 +402,10 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>"pending"</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>"unread"</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>audit_log</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>TRUE</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -451,10 +434,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>NULL for system default categories</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>expense_categories(id) ON DELETE RESTRICT</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -471,22 +450,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">users(id) ON DELETE </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="等线"/>
-        <family val="3"/>
-        <charset val="134"/>
-      </rPr>
-      <t>SET NULL</t>
-    </r>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Composite Unique</t>
   </si>
   <si>
@@ -525,10 +488,6 @@
   </si>
   <si>
     <t>user_role IN ("user", "admin")</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>status IN ("pending","accepted","revoked","expired")</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -581,10 +540,6 @@
   </si>
   <si>
     <t>account_book_id</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>ADD CONSTRAINT unique_account_user UNIQUE (account_book_id, user_id);</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -727,26 +682,6 @@
   </si>
   <si>
     <t>4</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>5</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>6</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>7</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>8</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>9</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -826,10 +761,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>ip_add</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>11</t>
   </si>
   <si>
@@ -846,10 +777,6 @@
   </si>
   <si>
     <t>example: #4CAF50</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>color IN (color ~ '^#[0-9A-Fa-f]{6}$')</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -979,12 +906,167 @@
     <t xml:space="preserve">avatar_path </t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
+  <si>
+    <t>not the only source truth</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>the only source truth</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t xml:space="preserve">CREATE UNIQUE INDEX cuq_accountbook_owner ON accountbook_user_permissions(account_book_id) WHERE account_role = 'owner';    </t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="等线"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>active</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Yu Gothic"/>
+        <family val="2"/>
+        <charset val="128"/>
+      </rPr>
+      <t>"</t>
+    </r>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>status IN ("active","revoked","expired")</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>account_role IN ("viewer","editor","admin")</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>max_usage &gt; 0 AND used_count &gt;= 0 AND used_count &lt;= max_usage</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>is_system_seed</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FALSE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>cuq_expense_categories_accountbook_name</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>color ~ '^#[0-9A-Fa-f]{6}$'</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>NULL only when user is hard deleted</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CURRENT_DATE</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CREATE INDEX idx_expenses_account_book_id_spent_at ON expenses(account_book_id, spent_at);</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(cycle_type = 'week' AND cycle_start_day BETWEEN 1 AND 7) OR (cycle_type = 'month' AND cycle_start_day BETWEEN 1 AND 28)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ip_address</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>latency_ms</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>numeric(10,3)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>action</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_id</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>target_type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>detail</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>jsonb</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>category_templates</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>request_logs</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>audit_events</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1073,6 +1155,34 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="等线"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Yu Gothic"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1094,7 +1204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1117,6 +1227,9 @@
     <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1398,7 +1511,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
@@ -1448,19 +1561,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1477,7 +1590,7 @@
         <v>13</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>15</v>
@@ -1543,7 +1656,7 @@
       </c>
       <c r="H7" s="3"/>
       <c r="L7" s="1" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -1551,7 +1664,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>17</v>
@@ -1560,10 +1673,10 @@
         <v>14</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="M8" s="3"/>
     </row>
@@ -1572,7 +1685,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>12</v>
@@ -1584,7 +1697,7 @@
         <v>13</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -1592,13 +1705,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>172</v>
+        <v>156</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>29</v>
@@ -1615,7 +1728,7 @@
         <v>23</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H11" s="1" t="b">
         <v>1</v>
@@ -1670,11 +1783,6 @@
       </c>
       <c r="H14" s="1" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" s="1" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>
@@ -1696,6 +1804,241 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1012007D-ABCC-4F8F-8F9F-B56C0C7D7726}">
+  <sheetPr codeName="Sheet9"/>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="7" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="19" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="32.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="52.109375" style="1" customWidth="1"/>
+    <col min="13" max="13" width="29" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A4" s="4">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A5" s="4">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A6" s="4">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A7" s="4">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+    </row>
+    <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A8" s="4">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>78</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="M8" s="6" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A9" s="4">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A11" s="2"/>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3715C3DB-8EE6-4A3A-A953-77AC433F117B}">
+          <x14:formula1>
+            <xm:f>temp!$A$1:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>D1:G1048576 I1:I1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{ACBC8FAF-88B3-4438-8C45-A099C91A945B}">
   <sheetPr codeName="Sheet10"/>
   <dimension ref="A1:M8"/>
@@ -1719,7 +2062,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1748,19 +2091,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -1788,7 +2131,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -1799,17 +2142,17 @@
       <c r="F4" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="J4" s="2" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2"/>
       <c r="M4" s="1" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -1817,7 +2160,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>17</v>
@@ -1825,9 +2168,10 @@
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2" t="s">
-        <v>84</v>
-      </c>
+      <c r="G5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
@@ -1838,7 +2182,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>25</v>
@@ -1858,7 +2202,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>25</v>
@@ -1912,10 +2256,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F12163D-5FF5-4FF5-AEC5-4D9FC6B4F58F}">
   <sheetPr codeName="Sheet11"/>
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
@@ -1936,7 +2280,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>91</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -1965,19 +2309,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2002,58 +2346,54 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A5" s="4" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="E5" s="2"/>
       <c r="F5" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="J5" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="J5" s="2"/>
       <c r="K5" s="2"/>
       <c r="L5" s="2"/>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A6" s="4" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
@@ -2063,55 +2403,55 @@
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A7" s="4" t="s">
-        <v>149</v>
+        <v>167</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>17</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A8" s="4" t="s">
-        <v>150</v>
+        <v>168</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="C8" s="15" t="s">
         <v>17</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I8" s="13"/>
       <c r="J8" s="13"/>
       <c r="K8" s="13"/>
       <c r="L8" s="13"/>
       <c r="M8" s="1" t="s">
-        <v>162</v>
+        <v>148</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A9" s="4" t="s">
-        <v>151</v>
+        <v>169</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>163</v>
+        <v>149</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>17</v>
       </c>
       <c r="F9" s="2" t="s">
-        <v>62</v>
+        <v>81</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -2121,13 +2461,13 @@
     </row>
     <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A10" s="4" t="s">
-        <v>152</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>164</v>
+        <v>170</v>
+      </c>
+      <c r="B10" s="18" t="s">
+        <v>179</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>14</v>
@@ -2135,10 +2475,10 @@
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>153</v>
+        <v>181</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>17</v>
@@ -2149,34 +2489,51 @@
     </row>
     <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A12" s="4" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>166</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>17</v>
+        <v>180</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>183</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="I12" s="2"/>
+        <v>61</v>
+      </c>
     </row>
     <row r="13" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A13" s="4" t="s">
-        <v>165</v>
-      </c>
-      <c r="B13" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I13" s="2"/>
+    </row>
+    <row r="14" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A14" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B14" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H13" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H14" s="2" t="s">
         <v>26</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>81</v>
       </c>
     </row>
   </sheetData>
@@ -2197,7 +2554,268 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D84B353C-B04A-454C-A6EB-2A3EB7699BD9}">
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="7" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="19" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="31.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="27" style="1" customWidth="1"/>
+    <col min="13" max="13" width="29" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A5" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+    </row>
+    <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A6" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+    </row>
+    <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A7" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="6"/>
+    </row>
+    <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A8" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="M8" s="1" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A9" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="C9" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
+      <c r="K9" s="13"/>
+      <c r="L9" s="13"/>
+      <c r="M9" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A10" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="13" t="s">
+        <v>187</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="6"/>
+    </row>
+    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
+      <c r="A11" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{97AE0225-36B6-43D5-830A-279D01E9F7A1}">
+          <x14:formula1>
+            <xm:f>temp!$A$1:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>I1:I1048576 D1:G1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{59F19E97-55D1-4225-B4A5-117B229AA299}">
   <dimension ref="A1:M10"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
@@ -2220,7 +2838,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2249,19 +2867,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2299,11 +2917,11 @@
         <v>14</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J4" s="2"/>
       <c r="K4" s="13" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="L4" s="2"/>
     </row>
@@ -2312,10 +2930,10 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>14</v>
@@ -2331,23 +2949,23 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J6" s="2"/>
       <c r="K6" s="13" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="L6" s="14" t="s">
-        <v>171</v>
+        <v>155</v>
       </c>
       <c r="M6" s="6"/>
     </row>
@@ -2356,13 +2974,13 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
@@ -2375,16 +2993,16 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>23</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -2397,19 +3015,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>14</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2420,7 +3038,7 @@
         <v>24</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>14</v>
@@ -2447,7 +3065,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BCA4C1A2-6A07-4758-BB44-9FCA05D2D5DB}">
   <sheetPr codeName="Sheet12"/>
   <dimension ref="A2:A3"/>
@@ -2493,7 +3111,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2522,19 +3140,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="6" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2576,7 +3194,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -2588,10 +3206,13 @@
         <v>14</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>95</v>
+        <v>90</v>
+      </c>
+      <c r="M5" s="6" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2599,7 +3220,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>21</v>
@@ -2609,7 +3230,7 @@
       </c>
       <c r="H6" s="9"/>
       <c r="L6" s="6" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2623,7 +3244,7 @@
         <v>17</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -2691,7 +3312,7 @@
         <v>13</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2736,7 +3357,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2765,19 +3386,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -2805,7 +3426,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -2821,10 +3442,10 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2832,7 +3453,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -2848,10 +3469,10 @@
         <v>13</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>110</v>
+        <v>103</v>
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
@@ -2859,7 +3480,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -2868,10 +3489,13 @@
         <v>14</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
+      </c>
+      <c r="M6" s="1" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.25">
@@ -2893,12 +3517,12 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
-        <v>124</v>
+      <c r="A11" s="16" t="s">
+        <v>159</v>
       </c>
     </row>
   </sheetData>
@@ -2943,7 +3567,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -2972,19 +3596,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="6" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="6" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3012,7 +3636,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>12</v>
@@ -3023,8 +3647,11 @@
       <c r="F4" s="6" t="s">
         <v>14</v>
       </c>
+      <c r="I4" s="6" t="s">
+        <v>81</v>
+      </c>
       <c r="J4" s="6" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3032,7 +3659,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>12</v>
@@ -3044,7 +3671,7 @@
         <v>14</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3052,7 +3679,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="C6" s="7" t="s">
         <v>17</v>
@@ -3061,10 +3688,10 @@
         <v>14</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="L6" s="6" t="s">
-        <v>113</v>
+        <v>162</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3072,7 +3699,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>17</v>
@@ -3085,7 +3712,7 @@
       </c>
       <c r="H7" s="7"/>
       <c r="M7" s="7" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3093,7 +3720,7 @@
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>25</v>
@@ -3110,13 +3737,19 @@
         <v>7</v>
       </c>
       <c r="B9" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="C9" s="7" t="s">
-        <v>43</v>
-      </c>
       <c r="F9" s="6" t="s">
         <v>14</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>163</v>
+      </c>
+      <c r="L9" s="6" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3124,13 +3757,16 @@
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F10" s="6" t="s">
         <v>14</v>
+      </c>
+      <c r="H10" s="6" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3138,19 +3774,19 @@
         <v>9</v>
       </c>
       <c r="B11" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>46</v>
-      </c>
       <c r="F11" s="6" t="s">
         <v>14</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>89</v>
+        <v>160</v>
       </c>
       <c r="L11" s="6" t="s">
-        <v>116</v>
+        <v>161</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -3191,7 +3827,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{724E6A76-50B2-4CCD-B787-16C42FB3153F}">
   <sheetPr codeName="Sheet5"/>
-  <dimension ref="A1:M11"/>
+  <dimension ref="A1:M12"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
@@ -3201,8 +3837,8 @@
     <col min="8" max="8" width="19" style="1" customWidth="1"/>
     <col min="9" max="9" width="6.77734375" style="1" customWidth="1"/>
     <col min="10" max="10" width="39.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="23.88671875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" style="1" customWidth="1"/>
+    <col min="12" max="12" width="34.109375" style="1" customWidth="1"/>
     <col min="13" max="13" width="29" style="1" customWidth="1"/>
     <col min="14" max="16384" width="8.88671875" style="1"/>
   </cols>
@@ -3212,7 +3848,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3241,19 +3877,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3281,7 +3917,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -3290,16 +3926,16 @@
         <v>13</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="M4" s="1" t="s">
-        <v>99</v>
+        <v>92</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.25">
@@ -3315,6 +3951,9 @@
       <c r="F5" s="1" t="s">
         <v>14</v>
       </c>
+      <c r="K5" s="1" t="s">
+        <v>173</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
@@ -3335,7 +3974,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>23</v>
@@ -3352,19 +3991,19 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>167</v>
+        <v>152</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
@@ -3372,16 +4011,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>25</v>
+        <v>171</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>26</v>
+        <v>172</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
@@ -3389,7 +4028,7 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>25</v>
@@ -3406,16 +4045,33 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>34</v>
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="4">
+        <v>10</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -3437,9 +4093,233 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{335BC6C6-3066-4188-848A-28E0BE21562F}">
+  <dimension ref="A1:M10"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="11.77734375" style="1" customWidth="1"/>
+    <col min="4" max="7" width="8.88671875" style="1"/>
+    <col min="8" max="8" width="19" style="1" customWidth="1"/>
+    <col min="9" max="9" width="6.77734375" style="1" customWidth="1"/>
+    <col min="10" max="10" width="39.21875" style="1" customWidth="1"/>
+    <col min="11" max="11" width="17.109375" style="1" customWidth="1"/>
+    <col min="12" max="12" width="23.88671875" style="1" customWidth="1"/>
+    <col min="13" max="13" width="29" style="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H6" s="1" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>167</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F02BD9F9-ABC3-4CEF-B272-6E3F9782F06C}">
+          <x14:formula1>
+            <xm:f>temp!$A$1:$A$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>D1:G1048576 I1:I1048576</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{004A5237-2B0B-46E4-BBE1-F8A10B073376}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.21875" style="6" customWidth="1"/>
@@ -3460,7 +4340,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -3500,19 +4380,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -3547,7 +4427,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -3565,7 +4445,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="K4" s="1"/>
       <c r="L4" s="1"/>
@@ -3576,7 +4456,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -3586,24 +4466,28 @@
         <v>13</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>14</v>
+        <v>81</v>
       </c>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
-      <c r="I5" s="1"/>
+      <c r="I5" s="1" t="s">
+        <v>81</v>
+      </c>
       <c r="J5" s="1" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="K5" s="1"/>
       <c r="L5" s="1"/>
-      <c r="M5" s="1"/>
+      <c r="M5" s="1" t="s">
+        <v>175</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>12</v>
@@ -3621,7 +4505,7 @@
         <v>13</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="K6" s="1"/>
       <c r="L6" s="1"/>
@@ -3632,7 +4516,7 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>12</v>
@@ -3650,7 +4534,7 @@
         <v>13</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -3707,10 +4591,10 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" s="1" t="s">
         <v>52</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -3730,7 +4614,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>21</v>
@@ -3746,7 +4630,7 @@
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
       <c r="M11" s="1"/>
     </row>
@@ -3755,10 +4639,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C12" s="1" t="s">
         <v>55</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>56</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -3778,10 +4662,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -3801,10 +4685,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -3813,11 +4697,9 @@
       </c>
       <c r="G14" s="1"/>
       <c r="H14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>13</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -3890,13 +4772,23 @@
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="6" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="17" t="s">
+        <v>177</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -3916,7 +4808,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B9972B4B-BE0F-4574-8515-34B392C707F7}">
   <sheetPr codeName="Sheet7"/>
   <dimension ref="A1:M14"/>
@@ -3940,7 +4832,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -3969,19 +4861,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="L2" s="1" t="s">
         <v>105</v>
       </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -4009,7 +4901,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>12</v>
@@ -4024,7 +4916,7 @@
         <v>13</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4032,7 +4924,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>12</v>
@@ -4044,10 +4936,10 @@
         <v>13</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4055,7 +4947,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>17</v>
@@ -4064,10 +4956,10 @@
         <v>14</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="30" x14ac:dyDescent="0.45">
@@ -4075,19 +4967,22 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="F7" s="1" t="s">
         <v>61</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>62</v>
       </c>
       <c r="H7" s="1">
         <v>1</v>
       </c>
+      <c r="L7" s="1" t="s">
+        <v>178</v>
+      </c>
       <c r="M7" s="11" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4095,10 +4990,10 @@
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>14</v>
@@ -4109,16 +5004,16 @@
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>66</v>
-      </c>
       <c r="F9" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4135,7 +5030,7 @@
         <v>14</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4143,13 +5038,13 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4157,13 +5052,13 @@
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4218,10 +5113,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{24A62F57-0A20-4451-8AFC-694FBD9F2D76}">
   <sheetPr codeName="Sheet8"/>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
@@ -4242,7 +5137,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -4271,19 +5166,19 @@
         <v>9</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>107</v>
+        <v>100</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>106</v>
+        <v>99</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -4311,7 +5206,7 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>21</v>
@@ -4322,10 +5217,10 @@
       <c r="I4" s="2"/>
       <c r="J4" s="2"/>
       <c r="K4" s="2" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4333,7 +5228,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>21</v>
@@ -4344,10 +5239,10 @@
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
       <c r="K5" s="2" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
@@ -4355,16 +5250,16 @@
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C6" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="F6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="M6" s="11" t="s">
         <v>72</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="M6" s="11" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
@@ -4372,21 +5267,21 @@
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>14</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>26</v>
+        <v>176</v>
       </c>
       <c r="I7" s="2"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="L7" s="2"/>
     </row>
@@ -4408,14 +5303,7 @@
       </c>
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A11" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
-        <v>75</v>
-      </c>
+      <c r="A11" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
@@ -4433,239 +5321,4 @@
     </ext>
   </extLst>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1012007D-ABCC-4F8F-8F9F-B56C0C7D7726}">
-  <sheetPr codeName="Sheet9"/>
-  <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.21875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="19.109375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="14" style="1" customWidth="1"/>
-    <col min="4" max="7" width="8.88671875" style="1"/>
-    <col min="8" max="8" width="19" style="1" customWidth="1"/>
-    <col min="9" max="9" width="6.77734375" style="1" customWidth="1"/>
-    <col min="10" max="10" width="32.88671875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="17.6640625" style="1" customWidth="1"/>
-    <col min="12" max="12" width="52.109375" style="1" customWidth="1"/>
-    <col min="13" max="13" width="29" style="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="4">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A4" s="4">
-        <v>2</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="1" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A5" s="4">
-        <v>3</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="10" t="s">
-        <v>78</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2" t="s">
-        <v>120</v>
-      </c>
-      <c r="M5" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A6" s="4">
-        <v>4</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A7" s="4">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-    </row>
-    <row r="8" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A8" s="4">
-        <v>6</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>81</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H8" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="13" t="s">
-        <v>121</v>
-      </c>
-      <c r="M8" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A9" s="4">
-        <v>7</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H9" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
-      <c r="A11" s="2"/>
-    </row>
-  </sheetData>
-  <phoneticPr fontId="1" type="noConversion"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3715C3DB-8EE6-4A3A-A953-77AC433F117B}">
-          <x14:formula1>
-            <xm:f>temp!$A$1:$A$3</xm:f>
-          </x14:formula1>
-          <xm:sqref>D1:G1048576 I1:I1048576</xm:sqref>
-        </x14:dataValidation>
-      </x14:dataValidations>
-    </ext>
-  </extLst>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Add expense_type in expense table
expense_type is "normal","merged_parent" or "merged_child"
</commit_message>
<xml_diff>
--- a/documents/database/databases.xlsx
+++ b/documents/database/databases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/445c6c4e8400985e/win数据迁移/Projects/Expense Statistics App Project/documents/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="703" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF85CBA6-8540-4A6A-8708-14D2FF62399D}"/>
+  <xr:revisionPtr revIDLastSave="727" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24164DDF-588E-40FE-9CD1-83EB0B532D2E}"/>
   <bookViews>
-    <workbookView xWindow="12540" yWindow="924" windowWidth="20604" windowHeight="15804" firstSheet="11" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="7188" windowWidth="30288" windowHeight="15000" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_users" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="800" uniqueCount="192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="194">
   <si>
     <t>Table name：</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1004,10 +1004,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>CREATE INDEX idx_expenses_account_book_id_spent_at ON expenses(account_book_id, spent_at);</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>(cycle_type = 'week' AND cycle_start_day BETWEEN 1 AND 7) OR (cycle_type = 'month' AND cycle_start_day BETWEEN 1 AND 28)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -1059,6 +1055,18 @@
   </si>
   <si>
     <t>audit_events</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>expense_type</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CREATE INDEX idx_expenses_account_book_id_expense_type_spent_at ON expenses(account_book_id, expense_type, spent_at);</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>(expense_type IN ('normal', 'merged_parent') AND parent_id IS NULL) OR  (expense_type = 'merged_child' AND parent_id IS NOT NULL)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1204,7 +1212,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1230,6 +1238,7 @@
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -2280,7 +2289,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2464,7 +2473,7 @@
         <v>170</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>82</v>
@@ -2475,7 +2484,7 @@
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>83</v>
@@ -2492,10 +2501,10 @@
         <v>140</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>61</v>
@@ -2518,7 +2527,7 @@
     </row>
     <row r="14" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A14" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>24</v>
@@ -2577,7 +2586,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -2705,7 +2714,7 @@
         <v>167</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C7" s="15" t="s">
         <v>17</v>
@@ -2724,7 +2733,7 @@
         <v>168</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>17</v>
@@ -2741,7 +2750,7 @@
         <v>169</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C9" s="15" t="s">
         <v>12</v>
@@ -2763,10 +2772,10 @@
         <v>170</v>
       </c>
       <c r="B10" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="C10" s="15" t="s">
         <v>187</v>
-      </c>
-      <c r="C10" s="15" t="s">
-        <v>188</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>81</v>
@@ -2779,7 +2788,7 @@
     </row>
     <row r="11" spans="1:13" ht="18" x14ac:dyDescent="0.45">
       <c r="A11" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>24</v>
@@ -4115,7 +4124,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.25">
@@ -4319,7 +4328,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{004A5237-2B0B-46E4-BBE1-F8A10B073376}">
   <sheetPr codeName="Sheet6"/>
-  <dimension ref="A1:M21"/>
+  <dimension ref="A1:M22"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.21875" style="6" customWidth="1"/>
@@ -4516,28 +4525,24 @@
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>12</v>
+        <v>191</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>17</v>
       </c>
       <c r="D7" s="1"/>
-      <c r="E7" s="1" t="s">
-        <v>13</v>
-      </c>
+      <c r="E7" s="1"/>
       <c r="F7" s="1" t="s">
-        <v>13</v>
+        <v>61</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-      <c r="I7" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>95</v>
-      </c>
+      <c r="I7" s="1"/>
+      <c r="J7" s="1"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="1"/>
+      <c r="L7" s="19" t="s">
+        <v>193</v>
+      </c>
       <c r="M7" s="1"/>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.25">
@@ -4545,20 +4550,26 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>50</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>12</v>
       </c>
       <c r="D8" s="1"/>
-      <c r="E8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>13</v>
+      </c>
       <c r="F8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
-      <c r="I8" s="1"/>
-      <c r="J8" s="1"/>
+      <c r="I8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>95</v>
+      </c>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
@@ -4568,7 +4579,7 @@
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>17</v>
@@ -4576,7 +4587,7 @@
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="1"/>
@@ -4591,15 +4602,15 @@
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>51</v>
+        <v>10</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>52</v>
+        <v>17</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -4614,10 +4625,10 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>21</v>
+        <v>52</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -4629,9 +4640,7 @@
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
-      <c r="L11" s="1" t="s">
-        <v>119</v>
-      </c>
+      <c r="L11" s="1"/>
       <c r="M11" s="1"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -4639,10 +4648,10 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -4654,7 +4663,9 @@
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
-      <c r="L12" s="1"/>
+      <c r="L12" s="1" t="s">
+        <v>119</v>
+      </c>
       <c r="M12" s="1"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -4662,10 +4673,10 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -4685,10 +4696,10 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>121</v>
+        <v>56</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>52</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -4696,9 +4707,7 @@
         <v>14</v>
       </c>
       <c r="G14" s="1"/>
-      <c r="H14" s="1" t="s">
-        <v>176</v>
-      </c>
+      <c r="H14" s="1"/>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
@@ -4710,10 +4719,10 @@
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>25</v>
+        <v>121</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -4722,7 +4731,7 @@
       </c>
       <c r="G15" s="1"/>
       <c r="H15" s="1" t="s">
-        <v>26</v>
+        <v>176</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
@@ -4735,7 +4744,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>25</v>
@@ -4760,7 +4769,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>25</v>
@@ -4768,11 +4777,11 @@
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G17" s="1"/>
       <c r="H17" s="1" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -4780,14 +4789,39 @@
       <c r="L17" s="1"/>
       <c r="M17" s="1"/>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" s="6" t="s">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="4">
+        <v>16</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D18" s="1"/>
+      <c r="E18" s="1"/>
+      <c r="F18" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="1"/>
+      <c r="H18" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="1"/>
+      <c r="M18" s="1"/>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" s="17" t="s">
-        <v>177</v>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="17" t="s">
+        <v>192</v>
       </c>
     </row>
   </sheetData>
@@ -4979,7 +5013,7 @@
         <v>1</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="M7" s="11" t="s">
         <v>62</v>

</xml_diff>

<commit_message>
Add "language" to user table. Reflected in backend code.
  - POST /api/v1/identity/register now need 'language' as a param
  - PUT /api/v1/identity/me/profile now need 'language' as a param
  - returned user payload will include 'language'
</commit_message>
<xml_diff>
--- a/documents/database/databases.xlsx
+++ b/documents/database/databases.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/445c6c4e8400985e/win数据迁移/Projects/Expense Statistics App Project/documents/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="727" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{24164DDF-588E-40FE-9CD1-83EB0B532D2E}"/>
+  <xr:revisionPtr revIDLastSave="737" documentId="8_{8ADEEE24-66C5-4752-B089-7156A878934A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E73E14B4-580E-4E3B-B314-92C023D0DF16}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="7188" windowWidth="30288" windowHeight="15000" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9204" yWindow="1356" windowWidth="21024" windowHeight="15000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01_users" sheetId="1" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="809" uniqueCount="197">
   <si>
     <t>Table name：</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -1067,6 +1067,18 @@
   </si>
   <si>
     <t>(expense_type IN ('normal', 'merged_parent') AND parent_id IS NULL) OR  (expense_type = 'merged_child' AND parent_id IS NOT NULL)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>language</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>"zh-CN"</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>language IN ('zh-CN', 'en', 'ja')</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -1212,7 +1224,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1238,7 +1250,6 @@
     <xf numFmtId="49" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1520,7 +1531,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.33203125" style="1" customWidth="1"/>
@@ -1673,57 +1684,60 @@
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>194</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>14</v>
+        <v>61</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>84</v>
+        <v>195</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="M8" s="3"/>
+        <v>196</v>
+      </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="J9" s="1" t="s">
-        <v>88</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="M9" s="3"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>156</v>
+        <v>114</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>17</v>
+        <v>12</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.25">
@@ -1731,16 +1745,16 @@
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>22</v>
+        <v>156</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H11" s="1" t="b">
-        <v>1</v>
+        <v>81</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.25">
@@ -1748,16 +1762,16 @@
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>25</v>
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>23</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H12" s="1" t="s">
-        <v>26</v>
+        <v>61</v>
+      </c>
+      <c r="H12" s="1" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.25">
@@ -1765,7 +1779,7 @@
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>25</v>
@@ -1782,15 +1796,32 @@
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>25</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H14" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="4">
+        <v>13</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" s="1" t="s">
         <v>29</v>
       </c>
     </row>
@@ -4540,7 +4571,7 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="19" t="s">
+      <c r="L7" s="1" t="s">
         <v>193</v>
       </c>
       <c r="M7" s="1"/>

</xml_diff>